<commit_message>
📊 Horarios actualizados Línea 141 - 5024
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-03.xlsx
+++ b/data/horarios-141-2026-10-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:00:04</t>
+          <t>Última actualización: 10:06:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>10:07</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>10:12</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:47</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>61</v>
+        <v>20</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:09</t>
+          <t>10:42</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>69</v>
+        <v>36</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:13</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,12 +648,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>94</v>
+        <v>49</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>10:57</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>101</v>
+        <v>56</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:56</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>116</v>
+        <v>64</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,23 +798,223 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>11:12</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>66</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>67</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>79</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>81</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>92</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>94</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>96</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>119</v>
-      </c>
-      <c r="E19" t="inlineStr">
+      <c r="D26" t="n">
+        <v>106</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>11:57</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>111</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -844,7 +1044,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:00:04</t>
+          <t>Última actualización: 10:06:58</t>
         </is>
       </c>
     </row>
@@ -885,21 +1085,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:13</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -910,21 +1110,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:00:04</t>
+          <t>10:06:58</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06:56</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -943,7 +1143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -956,14 +1156,141 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:00:04</t>
+          <t>Última actualización: 10:06:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>21</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>28</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>10:06:58</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>81</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5025
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-03.xlsx
+++ b/data/horarios-141-2026-10-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:06:58</t>
+          <t>Última actualización: 14:12:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -1015,6 +1015,531 @@
         <v>111</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>13</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>14</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>16</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>29</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>36</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>43</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>44</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>55</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>55</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>59</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>61</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>74</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>76</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>89</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>96</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>104</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>104</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>115</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>118</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1031,7 +1556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1044,14 +1569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:06:58</t>
+          <t>Última actualización: 14:12:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1127,6 +1652,106 @@
         <v>92</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>16</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>36</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>44</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>76</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1143,7 +1768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1156,14 +1781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:06:58</t>
+          <t>Última actualización: 14:12:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1289,6 +1914,81 @@
         <v>81</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>16</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>61</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>14:12:29</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>101</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5026
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-03.xlsx
+++ b/data/horarios-141-2026-10-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:12:30</t>
+          <t>Última actualización: 16:51:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 63</t>
         </is>
       </c>
     </row>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1540,6 +1540,506 @@
         <v>118</v>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>4</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>5</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>17</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>31</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>34</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>40</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>41</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>45</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>47</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>59</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>62</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>74</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>77</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>79</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>89</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>89</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>92</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>104</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>106</v>
+      </c>
+      <c r="E68" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1556,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1569,14 +2069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:12:30</t>
+          <t>Última actualización: 16:51:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1752,6 +2252,106 @@
         <v>76</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>17</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>41</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>62</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>92</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1768,7 +2368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1781,14 +2381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:12:30</t>
+          <t>Última actualización: 16:51:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1989,6 +2589,56 @@
         <v>101</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>17:02</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>11</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>16:51:36</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>18:29</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>98</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5027
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-03.xlsx
+++ b/data/horarios-141-2026-10-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:51:36</t>
+          <t>Última actualización: 19:29:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 63</t>
+          <t>Total filas: 80</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2040,6 +2040,431 @@
         <v>106</v>
       </c>
       <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>11</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>12</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>14</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>26</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>32</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>33</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>41</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>53</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>20:24</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>55</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>71</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>72</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>75</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>82</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>93</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>93</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>21:09</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>100</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>117</v>
+      </c>
+      <c r="E85" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2056,7 +2481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2069,14 +2494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:51:36</t>
+          <t>Última actualización: 19:29:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2352,6 +2777,56 @@
         <v>92</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>41</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>72</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2368,7 +2843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2381,14 +2856,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:51:36</t>
+          <t>Última actualización: 19:29:46</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2639,6 +3114,56 @@
         <v>98</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>32</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>19:29:46</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>72</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5028
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-03.xlsx
+++ b/data/horarios-141-2026-10-03.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:46</t>
+          <t>Última actualización: 22:50:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 80</t>
+          <t>Total filas: 85</t>
         </is>
       </c>
     </row>
@@ -2465,6 +2465,131 @@
         <v>117</v>
       </c>
       <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>22:50:16</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>23:04</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>14</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>22:50:16</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>23:19</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>29</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>22:50:16</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>23:37</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>47</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>22:50:16</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>50</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>22:50:16</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>23:59</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>69</v>
+      </c>
+      <c r="E90" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2481,7 +2606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2494,14 +2619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:46</t>
+          <t>Última actualización: 22:50:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2827,6 +2952,31 @@
         <v>72</v>
       </c>
       <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>22:50:16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>23:40</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>50</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2856,7 +3006,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:29:46</t>
+          <t>Última actualización: 22:50:16</t>
         </is>
       </c>
     </row>

</xml_diff>